<commit_message>
Add Task Tracker sheet — clean 2-color design with auto-status
- 50-row task list: Task Description, Assigned To, Check, Status columns
- Wide columns (46/24/12/18) for easy reading and entry
- 2 colors only: dark navy header + white/light-grey alternating rows
- Check column: tap to toggle (x14 native checkbox in Excel 365)
  - Empty rows stay neutral; fills red only when task exists + unchecked
  - Turns green on check
- Status auto-formula: blank when row empty; Complete (green) or
  In Progress (soft orange) based on Check value
- Includes x14 checkbox injection and Google Sheets Apps Script entry

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rAQaPAXkFohZahmsExXoT
</commit_message>
<xml_diff>
--- a/Personal_Life_Tracker.xlsx
+++ b/Personal_Life_Tracker.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Expense &amp; Savings" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Goals &amp; Settings" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Monthly Summary" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Task Tracker" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Salat Tracker'!$A$3:$J$368</definedName>
@@ -24,6 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Steps Tracker'!$A$3:$G$368</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Running Tracker'!$A$3:$I$368</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Expense &amp; Savings'!$A$3:$I$368</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Task Tracker'!$A$3:$D$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -41,7 +43,7 @@
     <numFmt numFmtId="170" formatCode=";;;"/>
     <numFmt numFmtId="171" formatCode="+#,##0;-#,##0;0"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -214,8 +216,14 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00757575"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -317,6 +325,11 @@
         <fgColor rgb="00FFFDE7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECEFF1"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -344,7 +357,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -598,11 +611,14 @@
     <xf numFmtId="4" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="13">
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -712,6 +728,29 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFEBEE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <color rgb="00B71C1C"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFCDD2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00E65100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF3E0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1972,6 +2011,643 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00757575"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="38" customHeight="1">
+      <c r="A1" s="37" t="inlineStr">
+        <is>
+          <t>☑  TASK TRACKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="85" t="inlineStr">
+        <is>
+          <t>Tap Check ✓ to mark complete  •  Status updates automatically</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="67" t="inlineStr">
+        <is>
+          <t>Task Description</t>
+        </is>
+      </c>
+      <c r="B3" s="67" t="inlineStr">
+        <is>
+          <t>Assigned To</t>
+        </is>
+      </c>
+      <c r="C3" s="67" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="D3" s="67" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="40" t="inlineStr"/>
+      <c r="B4" s="40" t="inlineStr"/>
+      <c r="C4" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="40">
+        <f>IF(A4="","",IF(C4=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="44" t="inlineStr"/>
+      <c r="B5" s="44" t="inlineStr"/>
+      <c r="C5" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="44">
+        <f>IF(A5="","",IF(C5=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="40" t="inlineStr"/>
+      <c r="B6" s="40" t="inlineStr"/>
+      <c r="C6" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="40">
+        <f>IF(A6="","",IF(C6=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="44" t="inlineStr"/>
+      <c r="B7" s="44" t="inlineStr"/>
+      <c r="C7" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="44">
+        <f>IF(A7="","",IF(C7=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="40" t="inlineStr"/>
+      <c r="B8" s="40" t="inlineStr"/>
+      <c r="C8" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="40">
+        <f>IF(A8="","",IF(C8=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="44" t="inlineStr"/>
+      <c r="B9" s="44" t="inlineStr"/>
+      <c r="C9" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="44">
+        <f>IF(A9="","",IF(C9=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="40" t="inlineStr"/>
+      <c r="B10" s="40" t="inlineStr"/>
+      <c r="C10" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="40">
+        <f>IF(A10="","",IF(C10=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="44" t="inlineStr"/>
+      <c r="B11" s="44" t="inlineStr"/>
+      <c r="C11" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="44">
+        <f>IF(A11="","",IF(C11=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="40" t="inlineStr"/>
+      <c r="B12" s="40" t="inlineStr"/>
+      <c r="C12" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="40">
+        <f>IF(A12="","",IF(C12=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="44" t="inlineStr"/>
+      <c r="B13" s="44" t="inlineStr"/>
+      <c r="C13" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="44">
+        <f>IF(A13="","",IF(C13=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="40" t="inlineStr"/>
+      <c r="B14" s="40" t="inlineStr"/>
+      <c r="C14" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="40">
+        <f>IF(A14="","",IF(C14=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="44" t="inlineStr"/>
+      <c r="B15" s="44" t="inlineStr"/>
+      <c r="C15" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="44">
+        <f>IF(A15="","",IF(C15=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="40" t="inlineStr"/>
+      <c r="B16" s="40" t="inlineStr"/>
+      <c r="C16" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="40">
+        <f>IF(A16="","",IF(C16=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="44" t="inlineStr"/>
+      <c r="B17" s="44" t="inlineStr"/>
+      <c r="C17" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="44">
+        <f>IF(A17="","",IF(C17=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="40" t="inlineStr"/>
+      <c r="B18" s="40" t="inlineStr"/>
+      <c r="C18" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="40">
+        <f>IF(A18="","",IF(C18=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="44" t="inlineStr"/>
+      <c r="B19" s="44" t="inlineStr"/>
+      <c r="C19" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="44">
+        <f>IF(A19="","",IF(C19=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="40" t="inlineStr"/>
+      <c r="B20" s="40" t="inlineStr"/>
+      <c r="C20" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="40">
+        <f>IF(A20="","",IF(C20=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="44" t="inlineStr"/>
+      <c r="B21" s="44" t="inlineStr"/>
+      <c r="C21" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="44">
+        <f>IF(A21="","",IF(C21=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="40" t="inlineStr"/>
+      <c r="B22" s="40" t="inlineStr"/>
+      <c r="C22" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="40">
+        <f>IF(A22="","",IF(C22=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="44" t="inlineStr"/>
+      <c r="B23" s="44" t="inlineStr"/>
+      <c r="C23" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="44">
+        <f>IF(A23="","",IF(C23=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="40" t="inlineStr"/>
+      <c r="B24" s="40" t="inlineStr"/>
+      <c r="C24" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="40">
+        <f>IF(A24="","",IF(C24=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="44" t="inlineStr"/>
+      <c r="B25" s="44" t="inlineStr"/>
+      <c r="C25" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="44">
+        <f>IF(A25="","",IF(C25=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="40" t="inlineStr"/>
+      <c r="B26" s="40" t="inlineStr"/>
+      <c r="C26" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="40">
+        <f>IF(A26="","",IF(C26=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="44" t="inlineStr"/>
+      <c r="B27" s="44" t="inlineStr"/>
+      <c r="C27" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="44">
+        <f>IF(A27="","",IF(C27=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="A28" s="40" t="inlineStr"/>
+      <c r="B28" s="40" t="inlineStr"/>
+      <c r="C28" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="40">
+        <f>IF(A28="","",IF(C28=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="44" t="inlineStr"/>
+      <c r="B29" s="44" t="inlineStr"/>
+      <c r="C29" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="44">
+        <f>IF(A29="","",IF(C29=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="26" customHeight="1">
+      <c r="A30" s="40" t="inlineStr"/>
+      <c r="B30" s="40" t="inlineStr"/>
+      <c r="C30" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="40">
+        <f>IF(A30="","",IF(C30=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="44" t="inlineStr"/>
+      <c r="B31" s="44" t="inlineStr"/>
+      <c r="C31" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="44">
+        <f>IF(A31="","",IF(C31=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="40" t="inlineStr"/>
+      <c r="B32" s="40" t="inlineStr"/>
+      <c r="C32" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="40">
+        <f>IF(A32="","",IF(C32=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="A33" s="44" t="inlineStr"/>
+      <c r="B33" s="44" t="inlineStr"/>
+      <c r="C33" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="44">
+        <f>IF(A33="","",IF(C33=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="40" t="inlineStr"/>
+      <c r="B34" s="40" t="inlineStr"/>
+      <c r="C34" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="40">
+        <f>IF(A34="","",IF(C34=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="44" t="inlineStr"/>
+      <c r="B35" s="44" t="inlineStr"/>
+      <c r="C35" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="44">
+        <f>IF(A35="","",IF(C35=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="A36" s="40" t="inlineStr"/>
+      <c r="B36" s="40" t="inlineStr"/>
+      <c r="C36" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="40">
+        <f>IF(A36="","",IF(C36=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="26" customHeight="1">
+      <c r="A37" s="44" t="inlineStr"/>
+      <c r="B37" s="44" t="inlineStr"/>
+      <c r="C37" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="44">
+        <f>IF(A37="","",IF(C37=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="40" t="inlineStr"/>
+      <c r="B38" s="40" t="inlineStr"/>
+      <c r="C38" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="40">
+        <f>IF(A38="","",IF(C38=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="26" customHeight="1">
+      <c r="A39" s="44" t="inlineStr"/>
+      <c r="B39" s="44" t="inlineStr"/>
+      <c r="C39" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="44">
+        <f>IF(A39="","",IF(C39=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="26" customHeight="1">
+      <c r="A40" s="40" t="inlineStr"/>
+      <c r="B40" s="40" t="inlineStr"/>
+      <c r="C40" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="40">
+        <f>IF(A40="","",IF(C40=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="26" customHeight="1">
+      <c r="A41" s="44" t="inlineStr"/>
+      <c r="B41" s="44" t="inlineStr"/>
+      <c r="C41" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="44">
+        <f>IF(A41="","",IF(C41=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" ht="26" customHeight="1">
+      <c r="A42" s="40" t="inlineStr"/>
+      <c r="B42" s="40" t="inlineStr"/>
+      <c r="C42" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="40">
+        <f>IF(A42="","",IF(C42=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="26" customHeight="1">
+      <c r="A43" s="44" t="inlineStr"/>
+      <c r="B43" s="44" t="inlineStr"/>
+      <c r="C43" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="44">
+        <f>IF(A43="","",IF(C43=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="40" t="inlineStr"/>
+      <c r="B44" s="40" t="inlineStr"/>
+      <c r="C44" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="40">
+        <f>IF(A44="","",IF(C44=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="26" customHeight="1">
+      <c r="A45" s="44" t="inlineStr"/>
+      <c r="B45" s="44" t="inlineStr"/>
+      <c r="C45" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="44">
+        <f>IF(A45="","",IF(C45=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="26" customHeight="1">
+      <c r="A46" s="40" t="inlineStr"/>
+      <c r="B46" s="40" t="inlineStr"/>
+      <c r="C46" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="40">
+        <f>IF(A46="","",IF(C46=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="26" customHeight="1">
+      <c r="A47" s="44" t="inlineStr"/>
+      <c r="B47" s="44" t="inlineStr"/>
+      <c r="C47" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="44">
+        <f>IF(A47="","",IF(C47=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1">
+      <c r="A48" s="40" t="inlineStr"/>
+      <c r="B48" s="40" t="inlineStr"/>
+      <c r="C48" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="40">
+        <f>IF(A48="","",IF(C48=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="26" customHeight="1">
+      <c r="A49" s="44" t="inlineStr"/>
+      <c r="B49" s="44" t="inlineStr"/>
+      <c r="C49" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="44">
+        <f>IF(A49="","",IF(C49=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="26" customHeight="1">
+      <c r="A50" s="40" t="inlineStr"/>
+      <c r="B50" s="40" t="inlineStr"/>
+      <c r="C50" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="40">
+        <f>IF(A50="","",IF(C50=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="26" customHeight="1">
+      <c r="A51" s="44" t="inlineStr"/>
+      <c r="B51" s="44" t="inlineStr"/>
+      <c r="C51" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="44">
+        <f>IF(A51="","",IF(C51=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="26" customHeight="1">
+      <c r="A52" s="40" t="inlineStr"/>
+      <c r="B52" s="40" t="inlineStr"/>
+      <c r="C52" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="40">
+        <f>IF(A52="","",IF(C52=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="26" customHeight="1">
+      <c r="A53" s="44" t="inlineStr"/>
+      <c r="B53" s="44" t="inlineStr"/>
+      <c r="C53" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="44">
+        <f>IF(A53="","",IF(C53=1,"Complete","In Progress"))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:D53"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C4:C53">
+    <cfRule type="expression" priority="1" dxfId="11">
+      <formula>AND(A4&lt;&gt;"",C4=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>C4=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4:D53">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>D4="Complete"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="12">
+      <formula>D4="In Progress"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCF9B9E7-4FED-4B87-89B2-7A4E5FC3597B}">
+      <x14:dataValidations>
+        <x14:dataValidation type="checkBox">
+          <xm:sqref xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">C4:C53</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>